<commit_message>
Use "Vera Rubin" (two words) as the proper product name
The display name is "Vera Rubin", not "VeraRubin". Updates system_name,
accelerator_model_name and hw_notes in the system description JSON, and
NVIDIA's rows in summary.csv/json/xlsx.

This also matches how the MLPerf Inference v6.1 Supplemental Discussion
document refers to the platform.

Path/identifier tokens are unchanged and remain VR-NVL72_VR-288GB_aarch64x72_TRT.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/summary.xlsx
+++ b/summary.xlsx
@@ -536,7 +536,7 @@
   <dimension ref="A1:AN103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col hidden="1" min="2" max="3"/>
+    <col hidden="1" width="13" customWidth="1" min="2" max="3"/>
     <col width="9.140625" customWidth="1" style="1" min="18" max="101"/>
   </cols>
   <sheetData>
@@ -9132,7 +9132,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA VeraRubin NVL72 (72x VR-288GB_aarch64)</t>
+          <t>NVIDIA Vera Rubin NVL72 (72x VR-288GB_aarch64)</t>
         </is>
       </c>
       <c r="H101" s="2" t="n">
@@ -9148,7 +9148,7 @@
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA VeraRubin</t>
+          <t>NVIDIA Vera Rubin</t>
         </is>
       </c>
       <c r="L101" s="2" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA VeraRubin NVL72, 2300W TGP Per GPU</t>
+          <t>NVIDIA Vera Rubin NVL72, 2300W TGP Per GPU</t>
         </is>
       </c>
       <c r="P101" s="2">
@@ -9381,7 +9381,7 @@
   <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col hidden="1" min="2" max="3"/>
+    <col hidden="1" width="13" customWidth="1" min="2" max="3"/>
     <col width="9.140625" customWidth="1" style="1" min="18" max="101"/>
   </cols>
   <sheetData>
@@ -10395,7 +10395,7 @@
   <dimension ref="A1:Z16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col hidden="1" min="2" max="3"/>
+    <col hidden="1" width="13" customWidth="1" min="2" max="3"/>
     <col width="9.140625" customWidth="1" style="1" min="18" max="101"/>
   </cols>
   <sheetData>
@@ -11526,7 +11526,7 @@
   <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col hidden="1" min="2" max="3"/>
+    <col hidden="1" width="13" customWidth="1" min="2" max="3"/>
     <col width="9.140625" customWidth="1" style="1" min="18" max="101"/>
   </cols>
   <sheetData>

</xml_diff>